<commit_message>
Rebuild Golden Path BOQ+Project doc with SY Resort fixture (live-verified)
Replaces the "Hotel Lift Lobby" version, which was built before real Slab
stock existed (every line confirmed only via the no-stock warning popup).
This version uses the SY Resort fixture (BOQ0044 -> S00340 -> Project 37)
after a full real click-through, covering 5 things the old doc never
proved: real Select Slabs (+ new Auto-Select Slabs button), bulk Recompute
BOQ Prices, EGQ print showing real Slab dimensions, Milestone-reached
close-out, and the new Billing Stage target-amount column.

14 test cases across 7 categories, 7 real Playwright screenshots, updated
Excel export, library.html card/tree-link retitled.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-golden-path-boq-project-hotel.xlsx
+++ b/client-docs/test-cases/emg-o-golden-path-boq-project-hotel.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Golden Path BOQ+Project Hotel" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="GP BOQ+Project SY Resort" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -429,11 +429,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="32" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="40" customWidth="1" min="5" max="5"/>
@@ -487,17 +487,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-01</t>
+          <t>TC-SYR-01</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>1. เตรียม Rate ใหม่</t>
+          <t>1. เตรียม BOQ หลายวัสดุหลาย Zone</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>สร้าง Rate ผนัง ABSOLUTE BLACK (3 Cost Component)</t>
+          <t>เปิดเอกสาร BOQ ใหม่ ผูกลูกค้า SY Resort</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -507,20 +507,18 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>1. BOQ Estimation &gt; Rate Library &gt; New
-2. ตั้งรหัส/ชื่อ/หน่วย/สินค้าอ้างอิง
-3. เพิ่ม Cost Component 3 แถว: Material, Labour, Other</t>
+          <t>1. Contacts &gt; New &gt; ตั้งชื่อลูกค้า
+2. BOQ Estimation &gt; BOQ Documents &gt; New เลือกลูกค้า</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>[WALL-ABSBLK-2CM] ผนัง ABSOLUTE BLACK (หนา 2 ซม.)
-Material 3,450 + Labour 400 + Other 150 = 4,000 บาท/ตร.ม.</t>
+          <t>ลูกค้า = "SY Resort"</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Rate บันทึกสำเร็จ Total Rate/Unit = 4,000 บาท ตรงกับผลรวม 3 Component</t>
+          <t>เปิดฟอร์ม BOQ Document ใหม่ สถานะ Draft พร้อม Analytic Account ผูกอัตโนมัติ</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -532,170 +530,169 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-02</t>
+          <t>TC-SYR-02</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1. เตรียม Rate ใหม่</t>
+          <t>1. เตรียม BOQ หลายวัสดุหลาย Zone</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>สร้าง Rate พื้น SPIDER GREEN (3 Cost Component)</t>
+          <t>เพิ่ม 4 บรรทัด BOQ (ผนัง+พื้น x 2 Zone) พร้อม Duration/Milestone</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ทำ TC-SYR-01 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>1. ทำแบบเดียวกับ TC-BPH-01</t>
+          <t>1. เพิ่มบรรทัด เลือก Rate ผนัง ระบุ Zone/Qty/Duration
+2. เพิ่มบรรทัด เลือก Rate พื้น ระบุ Zone/Qty/Duration/Milestone
+3. ทำซ้ำอีกรอบสำหรับ Pool Deck</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>[FLOOR-SPGRN-2CM] พื้น SPIDER GREEN (หนา 2 ซม.)
-Material 3,850 + Labour 500 + Other 150 = 4,500 บาท/ตร.ม.</t>
+          <t>Lobby: ผนัง 12 ตร.ม.(4วัน)+พื้น 20 ตร.ม.(5วัน, Milestone lobby เสร็จ)
+Pool Deck: ผนัง 15 ตร.ม.(5วัน)+พื้น 25 ตร.ม.(6วัน, Milestone Pool Deck เสร็จ+ส่งมอบงาน)</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Rate Library มี 2 รายการใหม่ พร้อมใช้ในเอกสาร BOQ</t>
+          <t>4 BOQ Lines ราคา/หน่วยเติมอัตโนมัติจาก Rate — Amount Direct Cost รวม = 310,500 บาท</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-03</t>
+          <t>TC-SYR-03</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2. สร้าง BOQ หลายวัสดุหลาย Zone</t>
+          <t>1. เตรียม BOQ หลายวัสดุหลาย Zone</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>สร้างลูกค้าใหม่ + เปิดเอกสาร BOQ</t>
+          <t>ตั้ง Preliminaries 3% + Performance Security 5% ตรวจยอดรวม</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>ทำหมวด 1 เสร็จแล้ว</t>
+          <t>ทำ TC-SYR-02 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>1. Contacts &gt; New &gt; ตั้งชื่อบริษัท
-2. BOQ Estimation &gt; BOQ Documents &gt; New เลือกลูกค้า</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>ลูกค้า = "THE GRANDE VISTA HOTEL"</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>เปิดฟอร์ม BOQ Document ใหม่ สถานะ Draft พร้อม Analytic Account ผูกอัตโนมัติ</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TC-BPH-04</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>2. สร้าง BOQ หลายวัสดุหลาย Zone</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>เพิ่ม 6 บรรทัด BOQ (ผนัง+พื้น x 3 ชั้น) พร้อม Duration/Milestone</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-BPH-03 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>1. เพิ่มบรรทัด เลือก Rate ผนัง ระบุ Zone/Qty/Duration
-2. เพิ่มบรรทัด เลือก Rate พื้น ระบุ Zone/Qty/Duration/Milestone
-3. ทำซ้ำอีก 2 รอบสำหรับ L10/L11</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>L9/L10/L11: ผนัง 18 ตร.ม. + พื้น 9 ตร.ม. ต่อชั้น, Duration 6 วันทุกบรรทัด
-Milestone: L9/L10/L11 เสร็จ (L11 + ส่งมอบงาน)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>6 BOQ Lines ราคา/หน่วยเติมอัตโนมัติจาก Rate — Direct Cost รวม = 337,500 บาท</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>TC-BPH-05</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>2. สร้าง BOQ หลายวัสดุหลาย Zone</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>ตั้ง Preliminaries 3% + Performance Security 5% ตรวจยอดรวม</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-BPH-04 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>1. กรอก Preliminaries % = 3
 2. กรอก Performance Security % = 5
 3. Save ดูแถบสรุปยอด</t>
         </is>
       </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Preliminaries 3%, Performance Security 5%</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Direct Cost 310,500 + Preliminaries 9,315 + Overhead&amp;Profit 29,970 + Performance Security 15,525 = Amount Total 365,310 บาท</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>TC-SYR-04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2. ออกใบเสนอราคา + เปิดสวิตช์ Project</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>กด "สร้างใบเสนอราคา" (Generate Quotation)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-03 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม "สร้างใบเสนอราคา" บนหัว BOQ Document</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>ได้ใบเสนอราคาใหม่ S00340 มี Section คั่นทั้ง 2 Zone field BOQ Document ชี้กลับไป BOQ0044</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>TC-SYR-05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>2. ออกใบเสนอราคา + เปิดสวิตช์ Project</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>ติ๊ก "Sold as Project" + Confirm</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-04 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>1. แท็บ Other Info ติ๊ก "Sold as Project"
+2. กด Confirm</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Preliminaries 3%, Performance Security 5%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Direct Cost 337,500 + Preliminaries 10,125 + Overhead&amp;Profit 32,535 (9.64% ผสม) + Performance Security 16,875 = Total 397,035 บาท</t>
+          <t>SO ยืนยันสำเร็จ ยอดรวม 441,105.36 บาท (รวม VAT 7%) ระบบสร้าง Project + 4 Task ให้อัตโนมัติเบื้องหลัง</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -707,37 +704,38 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-06</t>
+          <t>TC-SYR-06</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>3. ออกใบเสนอราคา + เปิดสวิตช์ Project</t>
+          <t>3. เลือก Slab จริงจากสต๊อก</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>กด "สร้างใบเสนอราคา" (Generate Quotation)</t>
+          <t>กด Select Slabs บนบรรทัดผนัง Lobby ใช้ปุ่ม Auto-Select</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>ทำ TC-BPH-05 เสร็จแล้ว</t>
+          <t>ทำ TC-SYR-05 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม "สร้างใบเสนอราคา" บนหัว BOQ Document</t>
+          <t>1. บรรทัดผนัง Lobby กด "Select Slabs"
+2. กดปุ่ม "Auto-Select Slabs"</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ต้องการ 12.00 ตร.ม. ระบบเลือกให้ 3 แผ่น = 14.40 ตร.ม.</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>ได้ใบเสนอราคาใหม่ S00338 มี Section คั่นทั้ง 3 ชั้น field BOQ Document ชี้กลับไป BOQ0042</t>
+          <t>ระบบเลือก Slab จากสต๊อกจริงให้อัตโนมัติ 3 แผ่น พร้อมข้อความเตือน "พื้นที่ที่เลือกยังไม่ตรงกับที่ต้องการ (เลือกแล้ว 14.40 / ต้องการ 12.00 ตร.ม.)" (ไม่ใช่ error — Slab มีขนาดตายตัว)</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -749,71 +747,70 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-07</t>
+          <t>TC-SYR-07</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>3. ออกใบเสนอราคา + เปิดสวิตช์ Project</t>
+          <t>3. เลือก Slab จริงจากสต๊อก</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>ตรวจ Zone/ราคาต่อบรรทัดตรงกับ BOQ</t>
+          <t>ทำซ้ำครบทั้ง 4 บรรทัด ตรวจราคาอัปเดตจากจำนวน Slab จริง</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>ทำ TC-BPH-06 เสร็จแล้ว</t>
+          <t>ทำ TC-SYR-06 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1. เปิดแท็บ Order Lines ตรวจคอลัมน์ Zone/ราคาของทุกบรรทัด</t>
+          <t>1. ทำ Select Slabs ให้ครบทั้ง 4 บรรทัด
+2. ตรวจคอลัมน์ Slabs และ Quantity บนแต่ละบรรทัด</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>ผนัง Lobby 3 แผ่น x19,200=57,600 / พื้น Lobby 5 แผ่น x21,600=108,000 / ผนัง Pool Deck 4 แผ่น x19,200=76,800 / พื้น Pool Deck 5 แผ่น x21,600=108,000</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>6 บรรทัดจริง แต่ละบรรทัดมีปุ่ม "Select Slabs" คอลัมน์ Zone = L9/L10/L11 ตรงกับ BOQ Line เดิม</t>
+          <t>ทุกบรรทัดมีคอลัมน์ "Slabs" แสดงเลข Block+ขนาดจริง ราคาบรรทัดคำนวณจากจำนวนแผ่น x ราคาต่อแผ่น ไม่ใช่ตร.ม.เดิมจาก BOQ</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-08</t>
+          <t>TC-SYR-08</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>3. ออกใบเสนอราคา + เปิดสวิตช์ Project</t>
+          <t>4. Sync ราคา BOQ ให้ตรงต้นทุน Slab จริง</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>ติ๊ก "Sold as Project" + Confirm</t>
+          <t>กด Recompute BOQ Prices ปุ่มเดียวที่ header อัปเดตทุกบรรทัดพร้อมกัน</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>ทำ TC-BPH-07 เสร็จแล้ว</t>
+          <t>ทำ TC-SYR-07 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>1. แท็บ Other Info ติ๊ก "Sold as Project"
-2. กด Confirm
-3. เจอ popup เตือน กด "Confirm ต่อ"</t>
+          <t>1. กดปุ่ม "Recompute BOQ Prices" บนหัวใบสั่งขาย</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -823,39 +820,39 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>SO ยืนยันสำเร็จ ยอดรวม 424,827.45 บาท (รวม VAT 7%) ระบบสร้าง Project ให้อัตโนมัติเบื้องหลัง</t>
+          <t>บรรทัดสรุปยอด 3 บรรทัด (Preliminaries/Overhead&amp;Profit/Performance Security) คำนวณใหม่จาก Direct Cost จริงหลังเลือก Slab แถบเตือนราคาไม่ตรง (ถ้ามี) หายไป</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-09</t>
+          <t>TC-SYR-09</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>4. ตรวจ Project + Template งานมาตรฐาน</t>
+          <t>5. พิมพ์ใบเสนอราคาแสดงขนาด Slab จริง</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>เปิด Project ตรวจ 6 Task (2 ต่อ Zone)</t>
+          <t>กด "พิมพ์ใบเสนอราคา (EGQ)" ตรวจ PDF แสดงขนาด Slab จริง</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ทำ TC-BPH-08 เสร็จแล้ว</t>
+          <t>ทำ TC-SYR-08 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>1. กด smart button "Project" บนใบสั่งขาย</t>
+          <t>1. กดปุ่ม "พิมพ์ใบเสนอราคา (EGQ)" บนหัวใบสั่งขาย</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -865,138 +862,138 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Project "THE GRANDE VISTA HOTEL - S00338" มี 6 Task: ผนัง+พื้น x 3 Zone แต่ละ Task ผูก Zone ถูกต้อง</t>
+          <t>PDF แยกตาราง Zone ละ 1 ตาราง ใต้ชื่อสินค้าแต่ละบรรทัดโชว์เลข Block+ขนาด W x H x หนา=ตร.ม. ของทุกแผ่นที่เลือกจริง</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-10</t>
+          <t>TC-SYR-10</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>4. ตรวจ Project + Template งานมาตรฐาน</t>
+          <t>6. ตรวจ Project + Template + Milestone</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Apply Task Template Set "งานติดตั้งหน้างานมาตรฐาน (5 ขั้นตอน)" ให้ทุก Task</t>
+          <t>เปิด Task ตรวจฟิลด์ Zone/Origin Sale Line</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ทำ TC-BPH-09 เสร็จแล้ว</t>
+          <t>ทำ TC-SYR-05 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1. กด smart button "Project" บนใบสั่งขาย
+2. เปิด Task "พื้น SPIDER GREEN — 20 m²"</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>Project "SY Resort - S00340" มี 4 Task ผูก Zone ถูกต้อง Task ที่เปิดมี Zone=Lobby, Origin Sale Line Value=108,000 บาท ไม่มีฟิลด์ "Sales Order Item" ปรากฏ (ซ่อนแล้ว ไม่ได้ใช้งาน)</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-SYR-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>6. ตรวจ Project + Template + Milestone</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Apply Task Template Set ให้ทุก Task</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-10 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>1. เปิด Task แต่ละใบ กด "Apply Template"
 2. เลือก Template Set + วันเริ่ม
-3. ทำซ้ำครบทั้ง 6 Task</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
+3. ทำซ้ำครบทั้ง 4 Task</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>แต่ละ Task มี 5 Sub-task ย่อยจริง ("Sub-tasks 5/5" แสดงบนหัว Task)</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>แต่ละ Task มี 5 Sub-task ย่อยจริง ("Sub-tasks 5/5") วันที่ Planned เรียงต่อกันอัตโนมัติตาม Duration</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TC-BPH-11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>5. ปิดงานจริงครบ 3 Zone</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>ทำ Sub-task ทุกใบ + Task หลักให้ Done ครบทั้ง 3 Zone</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-BPH-10 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-SYR-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>6. ตรวจ Project + Template + Milestone</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>ปิด Sub-task+Task ทุกใบให้ Done ครบ 4 Task ตรวจ Milestone Reached</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-11 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>1. เปิดแต่ละ Sub-task ตั้งสถานะ Done ทีละใบ (5 ใบ/Task)
 2. ตั้ง Task หลักเป็น Done
-3. ทำซ้ำครบทั้ง 6 Task</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
+3. ทำซ้ำครบทั้ง 4 Task</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>ทุก Task ขึ้น "Done" พร้อมเครื่องหมายถูกสีเขียว การ์ดย้ายไปคอลัมน์ Done บน Kanban</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TC-BPH-12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>5. ปิดงานจริงครบ 3 Zone</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>ตรวจ Milestone ขึ้น "Reached" ครบทั้ง 3 Zone (จุดที่เจอบั๊กที่ 2)</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-BPH-11 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>1. เปิด Task "พื้น" ของแต่ละ Zone (ตัวถือ Milestone)
-2. ตรวจ field Milestone</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Milestone ทั้ง 3 (L9/L10/L11 เสร็จ) ขึ้นสถานะ Reached ถูกต้องทุกตัว</t>
+          <t>ทุก Task ขึ้น Done — Milestone ทั้ง 2 (lobby เสร็จ / Pool Deck เสร็จ+ส่งมอบงาน) ขึ้นสถานะ Reached ถูกต้องทุกตัว</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1008,40 +1005,38 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-13</t>
+          <t>TC-SYR-13</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>6. งานเพิ่มนอก BOQ + Billing Stage</t>
+          <t>7. ติดตาม Billing Stage ตาม Progress</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>PM เพิ่ม Task ใหม่ตรงบน Project สำหรับ Zone L12 (นอก BOQ เดิม)</t>
+          <t>กรอก Progress 35% + ตั้งเกณฑ์เก็บเงินงวดที่ 1 (30%) ตรวจยอดที่ควรวางบิล</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>ทำ TC-BPH-12 เสร็จแล้ว</t>
+          <t>ทำ TC-SYR-12 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>1. เพิ่มบรรทัดใหม่ในใบสั่งขาย S00338 (นอกรอบ BOQ เดิม)
-2. สร้าง Task ใหม่บน Project ผูก Zone + Sales Order Item
-3. ตั้งสถานะ In Progress</t>
+          <t>1. เปิด Task "พื้น SPIDER GREEN — 20 m²" กรอก Progress % = 35
+2. แท็บ Billing Stages เพิ่มแถวใหม่ "งวดที่ 1 (มัดจำ 30%)" เกณฑ์ 30%</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Zone = "L12 Lift Lobby (Extra Scope)"
-มูลค่า = 48,000 บาท (12 ตร.ม. x 4,000)</t>
+          <t>Origin Sale Line Value=108,000 บาท, เกณฑ์งวดที่ 1=30%</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Task ใหม่ขึ้นในคอลัมน์ "In Progress" field Origin Sale Line Value = 48,000 บาท</t>
+          <t>"ยอดที่ควรวางบิลงวดนี้"=32,400 บาท (30% x 108,000) — Is Reached (35&gt;=30) — ระบบโพสต์ chatter + สร้าง Activity ให้ PM</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1053,83 +1048,40 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>TC-BPH-14</t>
+          <t>TC-SYR-14</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>6. งานเพิ่มนอก BOQ + Billing Stage</t>
+          <t>7. ติดตาม Billing Stage ตาม Progress</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>กรอก Progress 50% + ตั้งเกณฑ์เก็บเงิน 2 งวด เห็นงวดแรกแจ้งเตือนอัตโนมัติ</t>
+          <t>PM กดยืนยันพร้อมเก็บเงินงวดที่ 1</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>ทำ TC-BPH-13 เสร็จแล้ว</t>
+          <t>ทำ TC-SYR-13 เสร็จแล้ว</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>1. กรอก Progress % = 50
-2. แท็บ Billing Stages เพิ่ม 2 แถว: งวดที่ 1 (เกณฑ์ 30%), งวดที่ 2 (เกณฑ์ 70%)</t>
+          <t>1. แท็บ Billing Stages แถวงวดที่ 1 กดปุ่ม "ยืนยันพร้อมเก็บเงิน"</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>งวดที่ 1 (มัดจำเริ่มงาน 30%) / งวดที่ 2 (กลางงาน 70%)</t>
+          <t>-</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>งวดที่ 1: Is Reached (50&gt;=30) / งวดที่ 2: ยังไม่ขึ้น (50&lt;70) — ระบบโพสต์ chatter + สร้าง Activity ให้ PM</t>
+          <t>งวดที่ 1: Confirmed พร้อมวันที่ยืนยัน — Activity เคลียร์อัตโนมัติ ยังต้องออก Invoice จริงผ่าน Down Payment wizard แยกต่างหาก</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>TC-BPH-15</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>6. งานเพิ่มนอก BOQ + Billing Stage</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>PM กดยืนยันพร้อมเก็บเงินงวดที่ 1</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-BPH-14 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>1. แท็บ Billing Stages แถวงวดที่ 1 กดปุ่ม "ยืนยันพร้อมเก็บเงิน"</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>งวดที่ 1: Confirmed พร้อมวันที่ยืนยัน — ยังต้องออก Invoice จริงผ่าน Down Payment wizard แยกต่างหาก</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>

<commit_message>
Golden Path: rewrite switch-BOQ doc (21 cases, new Marine Hotel fixture + Cut List), reorder SY Resort doc for price lock, note lock in Labor Cost TC-LC-10
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-golden-path-boq-project-hotel.xlsx
+++ b/client-docs/test-cases/emg-o-golden-path-boq-project-hotel.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H15"/>
+  <dimension ref="A1:H16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -492,7 +492,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>1. เตรียม BOQ หลายวัสดุหลาย Zone</t>
+          <t>1. เตรียม BOQ หลายวัสดุ หลาย Zone</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -535,12 +535,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1. เตรียม BOQ หลายวัสดุหลาย Zone</t>
+          <t>1. เตรียม BOQ หลายวัสดุ หลาย Zone</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>เพิ่ม 4 บรรทัด BOQ (ผนัง+พื้น x 2 Zone) พร้อม Duration/Milestone</t>
+          <t>เพิ่ม 4 บรรทัด BOQ (ผนัง+พื้น × 2 Zone) พร้อม Duration/Milestone</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -557,8 +557,7 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Lobby: ผนัง 12 ตร.ม.(4วัน)+พื้น 20 ตร.ม.(5วัน, Milestone lobby เสร็จ)
-Pool Deck: ผนัง 15 ตร.ม.(5วัน)+พื้น 25 ตร.ม.(6วัน, Milestone Pool Deck เสร็จ+ส่งมอบงาน)</t>
+          <t>Lobby: ผนัง 12 ตร.ม. (4 วัน) + พื้น 20 ตร.ม. (5 วัน, Milestone "lobby เสร็จ") Pool Deck: ผนัง 15 ตร.ม. (5 วัน) + พื้น 25 ตร.ม. (6 วัน, Milestone "Pool Deck เสร็จ + ส่งมอบงาน")</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
@@ -580,7 +579,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1. เตรียม BOQ หลายวัสดุหลาย Zone</t>
+          <t>1. เตรียม BOQ หลายวัสดุ หลาย Zone</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -649,7 +648,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>ได้ใบเสนอราคาใหม่ S00340 มี Section คั่นทั้ง 2 Zone field BOQ Document ชี้กลับไป BOQ0044</t>
+          <t>ได้ใบเสนอราคาใหม่ S00340 มี Section คั่นทั้ง 2 Zone field "BOQ Document" ชี้กลับไป BOQ0044</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -671,7 +670,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>ติ๊ก "Sold as Project" + Confirm</t>
+          <t>ติ๊กเปิดสวิตช์ "Sold as Project" (ยังไม่ Confirm)</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -682,7 +681,7 @@
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>1. แท็บ Other Info ติ๊ก "Sold as Project"
-2. กด Confirm</t>
+2. Save (ปล่อยสถานะเป็นใบเสนอราคา ยังไม่กด Confirm)</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
@@ -692,7 +691,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>SO ยืนยันสำเร็จ ยอดรวม 441,105.36 บาท (รวม VAT 7%) ระบบสร้าง Project + 4 Task ให้อัตโนมัติเบื้องหลัง</t>
+          <t>บันทึกสำเร็จ ใบยังเป็น Quotation (Draft) ยอดก่อนภาษี 365,310.00 บาท (รวม VAT 7% = 390,881.70) — บรรทัดหิน 4 บรรทัดยังเป็น จำนวน 1 × ราคาจาก BOQ (ผนัง Lobby 48,000 / พื้น Lobby 90,000 / ผนัง Pool Deck 60,000 / พื้น Pool Deck 112,500) บรรทัดสรุป 3 บรรทัด = 9,315 / 29,970 / 15,525</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -714,7 +713,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>กด Select Slabs บนบรรทัดผนัง Lobby ใช้ปุ่ม Auto-Select</t>
+          <t>กด "Select Slabs" บนบรรทัดผนัง Lobby ใช้ปุ่ม Auto-Select</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -735,7 +734,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>ระบบเลือก Slab จากสต๊อกจริงให้อัตโนมัติ 3 แผ่น พร้อมข้อความเตือน "พื้นที่ที่เลือกยังไม่ตรงกับที่ต้องการ (เลือกแล้ว 14.40 / ต้องการ 12.00 ตร.ม.)" (ไม่ใช่ error — Slab มีขนาดตายตัว)</t>
+          <t>ระบบเลือก Slab จากสต๊อกจริงให้อัตโนมัติ 3 แผ่น (BLK-26-0265 #7/#8/#9) พร้อมข้อความเตือน "พื้นที่ที่เลือกยังไม่ตรงกับที่ต้องการ (เลือกแล้ว 14.40 ตร.ม. / ต้องการ 12.00 ตร.ม.)"</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -757,7 +756,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>ทำซ้ำครบทั้ง 4 บรรทัด ตรวจราคาอัปเดตจากจำนวน Slab จริง</t>
+          <t>ทำซ้ำให้ครบทั้ง 4 บรรทัด ตรวจราคาอัปเดตจากจำนวน Slab จริง</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -767,18 +766,18 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>1. ทำ Select Slabs ให้ครบทั้ง 4 บรรทัด
+          <t>1. ทำ Select Slabs ให้ครบทั้ง 4 บรรทัด (ผนัง/พื้น × Lobby/Pool Deck)
 2. ตรวจคอลัมน์ Slabs และ Quantity บนแต่ละบรรทัด</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>ผนัง Lobby 3 แผ่น x19,200=57,600 / พื้น Lobby 5 แผ่น x21,600=108,000 / ผนัง Pool Deck 4 แผ่น x19,200=76,800 / พื้น Pool Deck 5 แผ่น x21,600=108,000</t>
+          <t>ผนัง Lobby 3 แผ่น×19,200=57,600 / พื้น Lobby 5 แผ่น×21,600=108,000 / ผนัง Pool Deck 4 แผ่น×19,200=76,800 / พื้น Pool Deck 5 แผ่น×21,600=108,000</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>ทุกบรรทัดมีคอลัมน์ "Slabs" แสดงเลข Block+ขนาดจริง ราคาบรรทัดคำนวณจากจำนวนแผ่น x ราคาต่อแผ่น ไม่ใช่ตร.ม.เดิมจาก BOQ</t>
+          <t>ทุกบรรทัดมีคอลัมน์ "Slabs" แสดงเลข Block+ขนาดจริงของทุกแผ่นที่เลือก ราคาบรรทัดคำนวณจากจำนวนแผ่น×ราคาต่อแผ่น ไม่ใช่ตร.ม.เดิมจาก BOQ · ยอดรวมใบก่อนภาษีขยับจาก 365,310.00 เป็น 405,210.00 (รวม VAT 7% = 433,574.70) เพราะ Slab จริงเกินพื้นที่ที่ BOQ ตั้งไว้ — ใบยังเป็น Draft จึงขยับตามได้ตามปกติ บรรทัดสรุป 3 บรรทัดยังเป็นค่าเดิม (9,315 / 29,970 / 15,525) รอ Sync ใน TC-SYR-08</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
@@ -800,7 +799,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>กด Recompute BOQ Prices ปุ่มเดียวที่ header อัปเดตทุกบรรทัดพร้อมกัน</t>
+          <t>Sync บรรทัดสรุปยอด 3 บรรทัดให้ตรงกับ Direct Cost จริง (ใช้ % เดิม)</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -810,7 +809,7 @@
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม "Recompute BOQ Prices" บนหัวใบสั่งขาย</t>
+          <t>1. ที่แถบเตือนใต้ตาราง Order Lines กดลิงก์ "Recompute จาก Slab จริง (ใช้ % เดิม)"</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
@@ -820,7 +819,7 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>บรรทัดสรุปยอด 3 บรรทัด (Preliminaries/Overhead&amp;Profit/Performance Security) คำนวณใหม่จาก Direct Cost จริงหลังเลือก Slab แถบเตือนราคาไม่ตรง (ถ้ามี) หายไป</t>
+          <t>บรรทัดสรุปยอด 3 บรรทัดคำนวณใหม่จาก Direct Cost จริง 405,210.00: Preliminaries (3%) = 10,512.00 · Project Management Fee = 33,816.00 · Performance Security (5%) = 17,520.00 · ยอดรวมใบก่อนภาษี = 412,248.00 (รวม VAT 7% = 441,105.36) · แถบเตือน "ราคายังไม่ตรงกับต้นทุนจริง" หายไป</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
@@ -837,12 +836,12 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>5. พิมพ์ใบเสนอราคาแสดงขนาด Slab จริง</t>
+          <t>5. ยืนยันใบสั่งขาย (ล็อกราคา) + พิมพ์ใบเสนอราคาแสดงขนาด Slab จริง</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>กด "พิมพ์ใบเสนอราคา (EGQ)" ตรวจ PDF แสดงขนาด Slab จริง</t>
+          <t>ยืนยันคำสั่งขาย (Confirm) ระบบสร้าง Project + 4 Task และล็อกยอดบรรทัดหิน</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -852,7 +851,9 @@
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>1. กดปุ่ม "พิมพ์ใบเสนอราคา (EGQ)" บนหัวใบสั่งขาย</t>
+          <t>1. กด Confirm บนใบสั่งขาย
+2. ถ้ามี popup เตือน ให้อ่านแล้วกด "Confirm ต่อ" (Slab เลือกครบแล้ว ปกติไม่ควรมีเตือนเรื่องสต๊อก)
+3. กดปุ่ม smart button "Project" ดูผลลัพธ์</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
@@ -862,12 +863,12 @@
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>PDF แยกตาราง Zone ละ 1 ตาราง ใต้ชื่อสินค้าแต่ละบรรทัดโชว์เลข Block+ขนาด W x H x หนา=ตร.ม. ของทุกแผ่นที่เลือกจริง</t>
+          <t>SO ยืนยันสำเร็จ (state = Sales Order) ยอดก่อนภาษี 412,248.00 (รวม VAT 7% = 441,105.36) ตรงกับก่อนกด Confirm เป๊ะ · ระบบสร้าง Project + 4 Task ให้อัตโนมัติ โดยมูลค่าของ Task (Origin Sale Line Value) เป็นยอดหลังเลือก Slab: ผนัง Lobby 57,600 · พื้น Lobby 108,000 · ผนัง Pool Deck 76,800 · พื้น Pool Deck 108,000</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
     </row>
@@ -879,164 +880,163 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>6. ตรวจ Project + Template + Milestone</t>
+          <t>5. ยืนยันใบสั่งขาย (ล็อกราคา) + พิมพ์ใบเสนอราคาแสดงขนาด Slab จริง</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
+          <t>กด "พิมพ์ใบเสนอราคา (EGQ)" ตรวจ PDF แสดงขนาด Slab จริง</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-09 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>1. กดปุ่ม "พิมพ์ใบเสนอราคา (EGQ)" บนหัวใบสั่งขาย</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>PDF แยกตาราง Zone ละ 1 ตาราง ใต้ชื่อสินค้าแต่ละบรรทัดโชว์เลข Block+ขนาด W×H×หนา=ตร.ม. ของทุกแผ่นที่เลือกจริง (เช่น "BLK-26-0265 #7 (3.00×1.60×0.020 ม. = 4.80 ตร.ม.)")</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>TC-SYR-11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>6. ตรวจ Project + ใส่ Template + ปิดงานจน Milestone Reached</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
           <t>เปิด Task ตรวจฟิลด์ Zone/Origin Sale Line</t>
         </is>
       </c>
-      <c r="D11" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-SYR-05 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-09 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>1. กด smart button "Project" บนใบสั่งขาย
 2. เปิด Task "พื้น SPIDER GREEN — 20 m²"</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Project "SY Resort - S00340" มี 4 Task ผูก Zone ถูกต้อง Task ที่เปิดมี Zone=Lobby, Origin Sale Line Value=108,000 บาท ไม่มีฟิลด์ "Sales Order Item" ปรากฏ (ซ่อนแล้ว ไม่ได้ใช้งาน)</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Project "SY Resort - S00340" มี 4 Task ผูก Zone ถูกต้อง Task ที่เปิดมี Zone = Lobby, Origin Sale Line ชี้กลับ S00340, Origin Sale Line Value = 108,000 บาท ไม่มีฟิลด์ "Sales Order Item" ปรากฏ</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>TC-SYR-11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>6. ตรวจ Project + Template + Milestone</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>TC-SYR-12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>6. ตรวจ Project + ใส่ Template + ปิดงานจน Milestone Reached</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
         <is>
           <t>Apply Task Template Set ให้ทุก Task</t>
         </is>
       </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-SYR-10 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-11 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
         <is>
           <t>1. เปิด Task แต่ละใบ กด "Apply Template"
 2. เลือก Template Set + วันเริ่ม
 3. ทำซ้ำครบทั้ง 4 Task</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>แต่ละ Task มี 5 Sub-task ย่อยจริง ("Sub-tasks 5/5") วันที่ Planned เรียงต่อกันอัตโนมัติตาม Duration</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>แต่ละ Task มี 5 Sub-task ย่อยจริง ("Sub-tasks 5/5" แสดงบนหัว Task) วันที่ Planned เรียงต่อกันอัตโนมัติตาม Duration</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>TC-SYR-12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>6. ตรวจ Project + Template + Milestone</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>ปิด Sub-task+Task ทุกใบให้ Done ครบ 4 Task ตรวจ Milestone Reached</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-SYR-11 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>TC-SYR-13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>6. ตรวจ Project + ใส่ Template + ปิดงานจน Milestone Reached</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>ปิด Sub-task+Task ทุกใบให้ Done ครบ 4 Task ตรวจ Milestone ขึ้น Reached</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-12 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>1. เปิดแต่ละ Sub-task ตั้งสถานะ Done ทีละใบ (5 ใบ/Task)
 2. ตั้ง Task หลักเป็น Done
 3. ทำซ้ำครบทั้ง 4 Task</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>ทุก Task ขึ้น Done — Milestone ทั้ง 2 (lobby เสร็จ / Pool Deck เสร็จ+ส่งมอบงาน) ขึ้นสถานะ Reached ถูกต้องทุกตัว</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>TC-SYR-13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>7. ติดตาม Billing Stage ตาม Progress</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>กรอก Progress 35% + ตั้งเกณฑ์เก็บเงินงวดที่ 1 (30%) ตรวจยอดที่ควรวางบิล</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-SYR-12 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>1. เปิด Task "พื้น SPIDER GREEN — 20 m²" กรอก Progress % = 35
-2. แท็บ Billing Stages เพิ่มแถวใหม่ "งวดที่ 1 (มัดจำ 30%)" เกณฑ์ 30%</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Origin Sale Line Value=108,000 บาท, เกณฑ์งวดที่ 1=30%</t>
-        </is>
-      </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>"ยอดที่ควรวางบิลงวดนี้"=32,400 บาท (30% x 108,000) — Is Reached (35&gt;=30) — ระบบโพสต์ chatter + สร้าง Activity ให้ PM</t>
+          <t>ทุก Task ขึ้น "Done" การ์ดย้ายไปคอลัมน์ Done บน Kanban — Milestone ทั้ง 2 ("lobby เสร็จ" / "Pool Deck เสร็จ + ส่งมอบงาน") ขึ้นสถานะ Reached ถูกต้องทุกตัว</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
@@ -1058,30 +1058,73 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
+          <t>กรอก Progress 35% + ตั้งเกณฑ์เก็บเงินงวดที่ 1 (30%) ตรวจ "ยอดที่ควรวางบิลงวดนี้"</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-13 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>1. เปิด Task "พื้น SPIDER GREEN — 20 m²" กรอก Progress % = 35
+2. แท็บ Billing Stages เพิ่มแถวใหม่: "งวดที่ 1 (มัดจำ 30%)" เกณฑ์ 30%</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Origin Sale Line Value = 108,000 บาท, เกณฑ์งวดที่ 1 = 30%</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>"ยอดที่ควรวางบิลงวดนี้" = 32,400 บาท (30% × 108,000) — "Is Reached" ✅ (เพราะ 35 ≥ 30) — ระบบโพสต์ chatter แจ้งเตือนอัตโนมัติ + สร้าง Activity ให้ PM</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>TC-SYR-15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>7. ติดตาม Billing Stage ตาม Progress</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
           <t>PM กดยืนยันพร้อมเก็บเงินงวดที่ 1</t>
         </is>
       </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>ทำ TC-SYR-13 เสร็จแล้ว</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>ทำ TC-SYR-14 เสร็จแล้ว</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>1. แท็บ Billing Stages แถวงวดที่ 1 กดปุ่ม "ยืนยันพร้อมเก็บเงิน"</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>งวดที่ 1: Confirmed พร้อมวันที่ยืนยัน — Activity เคลียร์อัตโนมัติ ยังต้องออก Invoice จริงผ่าน Down Payment wizard แยกต่างหาก</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>งวดที่ 1: "Confirmed" ✅ พร้อมวันที่ยืนยัน — Activity ของงวดนี้เคลียร์อัตโนมัติ (ยังต้องไปออก Invoice จริงผ่าน Down Payment wizard เองแยกต่างหาก ระบบไม่ออกบิลให้อัตโนมัติ)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>

</xml_diff>

<commit_message>
qa: SY Resort golden path re-run live (new screenshots TC-SYR-04..09); switch-BOQ notes from live run
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/client-docs/test-cases/emg-o-golden-path-boq-project-hotel.xlsx
+++ b/client-docs/test-cases/emg-o-golden-path-boq-project-hotel.xlsx
@@ -648,7 +648,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>ได้ใบเสนอราคาใหม่ S00340 มี Section คั่นทั้ง 2 Zone field "BOQ Document" ชี้กลับไป BOQ0044</t>
+          <t>ได้ใบเสนอราคาใหม่ S00413 มี Section คั่นทั้ง 2 Zone field "BOQ Document" ชี้กลับไป BOQ0090</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
@@ -734,7 +734,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>ระบบเลือก Slab จากสต๊อกจริงให้อัตโนมัติ 3 แผ่น (BLK-26-0265 #7/#8/#9) พร้อมข้อความเตือน "พื้นที่ที่เลือกยังไม่ตรงกับที่ต้องการ (เลือกแล้ว 14.40 ตร.ม. / ต้องการ 12.00 ตร.ม.)"</t>
+          <t>ระบบเลือก Slab จากสต๊อกจริงให้อัตโนมัติ 3 แผ่น (BLK-26-0265 #16/#17/#18) พร้อมข้อความเตือน "พื้นที่ที่เลือกยังไม่ตรงกับที่ต้องการ (เลือกแล้ว 14.40 ตร.ม. / ต้องการ 12.00 ตร.ม.)"</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">

</xml_diff>